<commit_message>
Rename 'maximum_overtime_hours' to 'maximum_overtime' across models, migrations, and views for consistency
</commit_message>
<xml_diff>
--- a/public/assets/excel/ot_plans.xlsx
+++ b/public/assets/excel/ot_plans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\hrms\public\assets\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCC81EE8-99B1-4FB9-A2D8-427F61DB12DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{705AEEE3-BBC6-468B-9D73-F046C1104AED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0CFE3684-D380-4965-BF50-73AA526BC3D1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{98BDCDA1-9A16-4958-9130-6EDB9F656944}"/>
   </bookViews>
   <sheets>
     <sheet name="ot_plans" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
     <t>Custom_Overtime_Rate</t>
   </si>
   <si>
-    <t>Maximum_Overtime_Hours</t>
+    <t>Maximum_Overtime_(minutes)</t>
   </si>
   <si>
     <t>Status</t>
@@ -948,7 +948,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC6E4BC5-6BC8-479D-870E-FFD464E8C3BE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B195C7B-681C-42AB-8245-140F0544F433}">
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>

</xml_diff>